<commit_message>
deploy: feature/careteam → branches/feature-careteam 2cc0336dfcd278593d953272ed99327f31ddf995
</commit_message>
<xml_diff>
--- a/branches/feature-careteam/CodeSystem-typ-av-careteam-cs.xlsx
+++ b/branches/feature-careteam/CodeSystem-typ-av-careteam-cs.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-15T08:56:04+00:00</t>
+    <t>2026-10-15T09:21:11+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,7 +84,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Kodverk som anger vilken typ av CareTeam som avses, till exempel fast kontakt eller vårdteam.</t>
+    <t>Kodverk som anger vilken typ av CareTeam som avses, till exempel fast kontakt eller vård- eller omsorgsteam.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -406,9 +406,7 @@
       <c r="A15" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="B15" t="s" s="2">
-        <v>13</v>
-      </c>
+      <c r="B15" s="2"/>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">

</xml_diff>